<commit_message>
Update Excel with Sheet 5: Branch 1 history
</commit_message>
<xml_diff>
--- a/branches_4_summary.xlsx
+++ b/branches_4_summary.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="g:\My Drive\ร้าน\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E65003-1482-4C55-97A3-B9D6A8331A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B74D791-70FE-41F2-9769-E45BC3F2350F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="20940" windowHeight="14020" activeTab="3" xr2:uid="{107E54F4-8403-47BA-9EEE-1006BFE8CC07}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="20940" windowHeight="14020" firstSheet="1" activeTab="4" xr2:uid="{107E54F4-8403-47BA-9EEE-1006BFE8CC07}"/>
   </bookViews>
   <sheets>
     <sheet name="สรุปภาพรวม" sheetId="1" r:id="rId1"/>
     <sheet name="รายรับรายจ่ายรายวัน_ก.ย.69" sheetId="2" r:id="rId2"/>
     <sheet name="ประวัติย้อนหลัง_สาขา4" sheetId="3" r:id="rId3"/>
     <sheet name="ประวัติย้อนหลัง_สาขา3" sheetId="4" r:id="rId4"/>
+    <sheet name="ประวัติย้อนหลัง_สาขา1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="114">
   <si>
     <t>รายงานสรุปผลประกอบการ ร้านลูกชิ้น (19 วันแรก กันยายน 2569)</t>
   </si>
@@ -334,6 +335,42 @@
   </si>
   <si>
     <t>เฉลี่ยต่อเดือน (9 เดือน)</t>
+  </si>
+  <si>
+    <t>สรุปประวัติผลประกอบการย้อนหลัง: สาขา 1 (มกราคม - กันยายน 2569)</t>
+  </si>
+  <si>
+    <t>ข้อมูลจากสมุดบัญชีรายวันยอดขายและรายจ่ายรายเดือน (9 เดือนสะสม - สาขาอันดับ 1 ทั้งรายรับและกำไรสุทธิ)</t>
+  </si>
+  <si>
+    <t>ทะลุเป้า 40k กำไรสุทธิสูงถึง +13,026 บ. (ค่าเช่า/ค่าไฟ 5,639 บ. วันที่ 6)</t>
+  </si>
+  <si>
+    <t>ขาย 28 วัน คุมรายจ่ายได้ดี จ่ายค่าเช่า 5,000 บ. วันที่ 2 กำไรสุทธิ +913 บ.</t>
+  </si>
+  <si>
+    <t>ยอดขายทะลุ 5.4 หมื่นบาท จ่ายค่าเช่า 5,000 บ. รวมค่าไฟตกค้าง 4,942 บ.</t>
+  </si>
+  <si>
+    <t>All-Time High! ยอดขายเทศกาลสงกรานต์ทะลุ 1.44 แสนบาท กำไรสุทธิ +45,056 บ.</t>
+  </si>
+  <si>
+    <t>ยอดขายเกิน 4.5 หมื่นบาท ทะลุเป้า 40k จ่ายค่าเช่า 5,000 บ. วันที่ 1</t>
+  </si>
+  <si>
+    <t>ยอดชะลอตัวตามฤดูกาล มีค่าเช่า 5,000 บ. และค่าไฟ 2,554 บ. วันที่ 1</t>
+  </si>
+  <si>
+    <t>ทะลุเป้า 40k ยอดพุ่ง 5.6 หมื่นบาท พลิกกลับมามีกำไรสุทธิ จ่ายค่าเช่า 5,000 บ.</t>
+  </si>
+  <si>
+    <t>ทะลุเป้า 40k ต่อเนื่อง กำไรสุทธิเด่น +4,333 บ. ทยอยเก็บค่าเช่าวันละ 215 บ.</t>
+  </si>
+  <si>
+    <t>ขาย 19 วัน กำไรดำเนินงานก่อนค่าเช่า +2,727 บ. คาดสิ้นเดือนแตะ ~31,140 บ.</t>
+  </si>
+  <si>
+    <t>ยอดขายและกำไรสุทธิอันดับ 1 ของทุกสาขา (กำไรสะสม +42,801 บ.)</t>
   </si>
 </sst>
 </file>
@@ -343,7 +380,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -390,8 +427,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF64748B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1E40AF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -428,6 +488,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDBEAFE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBFDBFE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -452,16 +530,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -490,6 +565,33 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -819,15 +921,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1881,17 +1983,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -2192,57 +2294,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="16" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="13">
         <v>2569</v>
       </c>
       <c r="C4" s="4">
@@ -2258,330 +2360,745 @@
         <v>4000</v>
       </c>
       <c r="G4" s="4">
+        <f t="shared" ref="G4:G14" si="0">D4-E4</f>
+        <v>11743</v>
+      </c>
+      <c r="H4" s="5">
+        <f t="shared" ref="H4:H14" si="1">G4/D4</f>
+        <v>0.15153431233385811</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C5" s="4">
+        <v>60000</v>
+      </c>
+      <c r="D5" s="4">
+        <v>44473</v>
+      </c>
+      <c r="E5" s="4">
+        <v>59117</v>
+      </c>
+      <c r="F5" s="4">
+        <v>4000</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="0"/>
+        <v>-14644</v>
+      </c>
+      <c r="H5" s="5">
+        <f t="shared" si="1"/>
+        <v>-0.32927843860319744</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C6" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D6" s="4">
+        <v>32186</v>
+      </c>
+      <c r="E6" s="4">
+        <v>40847</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2000</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="0"/>
+        <v>-8661</v>
+      </c>
+      <c r="H6" s="5">
+        <f t="shared" si="1"/>
+        <v>-0.26909215186727148</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C7" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D7" s="4">
+        <v>37470</v>
+      </c>
+      <c r="E7" s="4">
+        <v>38716</v>
+      </c>
+      <c r="F7" s="4">
+        <v>2000</v>
+      </c>
+      <c r="G7" s="4">
+        <f t="shared" si="0"/>
+        <v>-1246</v>
+      </c>
+      <c r="H7" s="5">
+        <f t="shared" si="1"/>
+        <v>-3.3253269282092338E-2</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C8" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D8" s="4">
+        <v>32214</v>
+      </c>
+      <c r="E8" s="4">
+        <v>29924</v>
+      </c>
+      <c r="F8" s="4">
+        <v>2000</v>
+      </c>
+      <c r="G8" s="4">
+        <f t="shared" si="0"/>
+        <v>2290</v>
+      </c>
+      <c r="H8" s="5">
+        <f t="shared" si="1"/>
+        <v>7.1087104985410071E-2</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C9" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D9" s="4">
+        <v>41143</v>
+      </c>
+      <c r="E9" s="4">
+        <v>49967</v>
+      </c>
+      <c r="F9" s="4">
+        <v>4000</v>
+      </c>
+      <c r="G9" s="4">
+        <f t="shared" si="0"/>
+        <v>-8824</v>
+      </c>
+      <c r="H9" s="5">
+        <f t="shared" si="1"/>
+        <v>-0.21447147752959192</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C10" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D10" s="4">
+        <v>49295</v>
+      </c>
+      <c r="E10" s="4">
+        <v>51785</v>
+      </c>
+      <c r="F10" s="4">
+        <v>2000</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" si="0"/>
+        <v>-2490</v>
+      </c>
+      <c r="H10" s="5">
+        <f t="shared" si="1"/>
+        <v>-5.0512222334922405E-2</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C11" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D11" s="4">
+        <v>45812</v>
+      </c>
+      <c r="E11" s="4">
+        <v>47343</v>
+      </c>
+      <c r="F11" s="4">
+        <v>2000</v>
+      </c>
+      <c r="G11" s="4">
+        <f t="shared" si="0"/>
+        <v>-1531</v>
+      </c>
+      <c r="H11" s="5">
+        <f t="shared" si="1"/>
+        <v>-3.3419191478215315E-2</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C12" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D12" s="4">
+        <v>27068</v>
+      </c>
+      <c r="E12" s="4">
+        <v>28119</v>
+      </c>
+      <c r="F12" s="4">
+        <v>4000</v>
+      </c>
+      <c r="G12" s="4">
+        <f t="shared" si="0"/>
+        <v>-1051</v>
+      </c>
+      <c r="H12" s="5">
+        <f t="shared" si="1"/>
+        <v>-3.8828136544997782E-2</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="9">
+        <f>SUM(D4:D12)</f>
+        <v>387155</v>
+      </c>
+      <c r="E13" s="9">
+        <f>SUM(E4:E12)</f>
+        <v>411569</v>
+      </c>
+      <c r="F13" s="9">
+        <f>SUM(F4:F12)</f>
+        <v>26000</v>
+      </c>
+      <c r="G13" s="9">
+        <f t="shared" si="0"/>
+        <v>-24414</v>
+      </c>
+      <c r="H13" s="11">
+        <f t="shared" si="1"/>
+        <v>-6.3060014722785454E-2</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="10">
+        <f>AVERAGE(D4:D12)</f>
+        <v>43017.222222222219</v>
+      </c>
+      <c r="E14" s="10">
+        <f>AVERAGE(E4:E12)</f>
+        <v>45729.888888888891</v>
+      </c>
+      <c r="F14" s="10">
+        <f>AVERAGE(F4:F12)</f>
+        <v>2888.8888888888887</v>
+      </c>
+      <c r="G14" s="10">
+        <f t="shared" si="0"/>
+        <v>-2712.6666666666715</v>
+      </c>
+      <c r="H14" s="12">
+        <f t="shared" si="1"/>
+        <v>-6.3060014722785565E-2</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E2F0F1-53F3-4849-A572-B467D0C617D8}">
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="85.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="69.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="19.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="22" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C4" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D4" s="4">
+        <v>44743</v>
+      </c>
+      <c r="E4" s="4">
+        <v>31717</v>
+      </c>
+      <c r="F4" s="4">
+        <v>5639</v>
+      </c>
+      <c r="G4" s="4">
         <f>D4-E4</f>
-        <v>11743</v>
+        <v>13026</v>
       </c>
       <c r="H4" s="5">
         <f>G4/D4</f>
-        <v>0.15153431233385811</v>
-      </c>
-      <c r="I4" s="18" t="s">
-        <v>82</v>
+        <v>0.29112933866750107</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="13">
         <v>2569</v>
       </c>
       <c r="C5" s="4">
-        <v>60000</v>
+        <v>40000</v>
       </c>
       <c r="D5" s="4">
-        <v>44473</v>
+        <v>31510</v>
       </c>
       <c r="E5" s="4">
-        <v>59117</v>
+        <v>30597</v>
       </c>
       <c r="F5" s="4">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="G5" s="4">
         <f>D5-E5</f>
-        <v>-14644</v>
+        <v>913</v>
       </c>
       <c r="H5" s="5">
         <f>G5/D5</f>
-        <v>-0.32927843860319744</v>
-      </c>
-      <c r="I5" s="18" t="s">
-        <v>84</v>
+        <v>2.8974928594097112E-2</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="13">
         <v>2569</v>
       </c>
       <c r="C6" s="4">
         <v>40000</v>
       </c>
       <c r="D6" s="4">
-        <v>32186</v>
+        <v>54373</v>
       </c>
       <c r="E6" s="4">
-        <v>40847</v>
+        <v>57267</v>
       </c>
       <c r="F6" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="G6" s="4">
         <f>D6-E6</f>
-        <v>-8661</v>
+        <v>-2894</v>
       </c>
       <c r="H6" s="5">
         <f>G6/D6</f>
-        <v>-0.26909215186727148</v>
-      </c>
-      <c r="I6" s="18" t="s">
-        <v>86</v>
+        <v>-5.3224946204917883E-2</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="13">
         <v>2569</v>
       </c>
       <c r="C7" s="4">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="D7" s="4">
-        <v>37470</v>
+        <v>144215</v>
       </c>
       <c r="E7" s="4">
-        <v>38716</v>
+        <v>99159</v>
       </c>
       <c r="F7" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="G7" s="4">
         <f>D7-E7</f>
-        <v>-1246</v>
+        <v>45056</v>
       </c>
       <c r="H7" s="5">
         <f>G7/D7</f>
-        <v>-3.3253269282092338E-2</v>
-      </c>
-      <c r="I7" s="18" t="s">
-        <v>88</v>
+        <v>0.31242242485178379</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="13">
         <v>2569</v>
       </c>
       <c r="C8" s="4">
         <v>40000</v>
       </c>
       <c r="D8" s="4">
-        <v>32214</v>
+        <v>45260</v>
       </c>
       <c r="E8" s="4">
-        <v>29924</v>
+        <v>47016</v>
       </c>
       <c r="F8" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="G8" s="4">
         <f>D8-E8</f>
-        <v>2290</v>
+        <v>-1756</v>
       </c>
       <c r="H8" s="5">
         <f>G8/D8</f>
-        <v>7.1087104985410071E-2</v>
-      </c>
-      <c r="I8" s="18" t="s">
-        <v>90</v>
+        <v>-3.8798055678303141E-2</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="13">
         <v>2569</v>
       </c>
       <c r="C9" s="4">
         <v>40000</v>
       </c>
       <c r="D9" s="4">
-        <v>41143</v>
+        <v>33265</v>
       </c>
       <c r="E9" s="4">
-        <v>49967</v>
+        <v>47218</v>
       </c>
       <c r="F9" s="4">
-        <v>4000</v>
+        <v>7554</v>
       </c>
       <c r="G9" s="4">
         <f>D9-E9</f>
-        <v>-8824</v>
+        <v>-13953</v>
       </c>
       <c r="H9" s="5">
         <f>G9/D9</f>
-        <v>-0.21447147752959192</v>
-      </c>
-      <c r="I9" s="18" t="s">
-        <v>92</v>
+        <v>-0.41944987223808811</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="13">
         <v>2569</v>
       </c>
       <c r="C10" s="4">
         <v>40000</v>
       </c>
       <c r="D10" s="4">
-        <v>49295</v>
+        <v>56370</v>
       </c>
       <c r="E10" s="4">
-        <v>51785</v>
+        <v>56021</v>
       </c>
       <c r="F10" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="G10" s="4">
         <f>D10-E10</f>
-        <v>-2490</v>
+        <v>349</v>
       </c>
       <c r="H10" s="5">
         <f>G10/D10</f>
-        <v>-5.0512222334922405E-2</v>
-      </c>
-      <c r="I10" s="18" t="s">
-        <v>94</v>
+        <v>6.1912364733014017E-3</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="13">
         <v>2569</v>
       </c>
       <c r="C11" s="4">
         <v>40000</v>
       </c>
       <c r="D11" s="4">
-        <v>45812</v>
+        <v>44005</v>
       </c>
       <c r="E11" s="4">
-        <v>47343</v>
+        <v>39672</v>
       </c>
       <c r="F11" s="4">
-        <v>2000</v>
+        <v>2150</v>
       </c>
       <c r="G11" s="4">
         <f>D11-E11</f>
-        <v>-1531</v>
+        <v>4333</v>
       </c>
       <c r="H11" s="5">
         <f>G11/D11</f>
-        <v>-3.3419191478215315E-2</v>
-      </c>
-      <c r="I11" s="18" t="s">
-        <v>96</v>
+        <v>9.8466083399613685E-2</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="13">
         <v>2569</v>
       </c>
       <c r="C12" s="4">
         <v>40000</v>
       </c>
       <c r="D12" s="4">
-        <v>27068</v>
+        <v>19720</v>
       </c>
       <c r="E12" s="4">
-        <v>28119</v>
+        <v>21993</v>
       </c>
       <c r="F12" s="4">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="G12" s="4">
         <f>D12-E12</f>
-        <v>-1051</v>
+        <v>-2273</v>
       </c>
       <c r="H12" s="5">
         <f>G12/D12</f>
-        <v>-3.8828136544997782E-2</v>
-      </c>
-      <c r="I12" s="18" t="s">
-        <v>98</v>
+        <v>-0.11526369168356998</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="24">
         <f>SUM(D4:D12)</f>
-        <v>387155</v>
-      </c>
-      <c r="E13" s="10">
+        <v>473461</v>
+      </c>
+      <c r="E13" s="24">
         <f>SUM(E4:E12)</f>
-        <v>411569</v>
-      </c>
-      <c r="F13" s="10">
+        <v>430660</v>
+      </c>
+      <c r="F13" s="24">
         <f>SUM(F4:F12)</f>
-        <v>26000</v>
-      </c>
-      <c r="G13" s="10">
+        <v>45343</v>
+      </c>
+      <c r="G13" s="24">
         <f>D13-E13</f>
-        <v>-24414</v>
-      </c>
-      <c r="H13" s="12">
+        <v>42801</v>
+      </c>
+      <c r="H13" s="26">
         <f>G13/D13</f>
-        <v>-6.3060014722785454E-2</v>
-      </c>
-      <c r="I13" s="19" t="s">
-        <v>100</v>
+        <v>9.0400265280561651E-2</v>
+      </c>
+      <c r="I13" s="31" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="25">
         <f>AVERAGE(D4:D12)</f>
-        <v>43017.222222222219</v>
-      </c>
-      <c r="E14" s="11">
+        <v>52606.777777777781</v>
+      </c>
+      <c r="E14" s="25">
         <f>AVERAGE(E4:E12)</f>
-        <v>45729.888888888891</v>
-      </c>
-      <c r="F14" s="11">
+        <v>47851.111111111109</v>
+      </c>
+      <c r="F14" s="25">
         <f>AVERAGE(F4:F12)</f>
-        <v>2888.8888888888887</v>
-      </c>
-      <c r="G14" s="11">
+        <v>5038.1111111111113</v>
+      </c>
+      <c r="G14" s="25">
         <f>D14-E14</f>
-        <v>-2712.6666666666715</v>
-      </c>
-      <c r="H14" s="13">
+        <v>4755.6666666666715</v>
+      </c>
+      <c r="H14" s="27">
         <f>G14/D14</f>
-        <v>-6.3060014722785565E-2</v>
-      </c>
-      <c r="I14" s="20" t="s">
+        <v>9.0400265280561734E-2</v>
+      </c>
+      <c r="I14" s="32" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel with Sheet 6: Annual Summary 2569
</commit_message>
<xml_diff>
--- a/branches_4_summary.xlsx
+++ b/branches_4_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="g:\My Drive\ร้าน\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B74D791-70FE-41F2-9769-E45BC3F2350F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{657439B9-B9BF-45A8-B59A-E4023917F16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="20940" windowHeight="14020" firstSheet="1" activeTab="4" xr2:uid="{107E54F4-8403-47BA-9EEE-1006BFE8CC07}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="20940" windowHeight="14020" firstSheet="2" activeTab="5" xr2:uid="{107E54F4-8403-47BA-9EEE-1006BFE8CC07}"/>
   </bookViews>
   <sheets>
     <sheet name="สรุปภาพรวม" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="ประวัติย้อนหลัง_สาขา4" sheetId="3" r:id="rId3"/>
     <sheet name="ประวัติย้อนหลัง_สาขา3" sheetId="4" r:id="rId4"/>
     <sheet name="ประวัติย้อนหลัง_สาขา1" sheetId="5" r:id="rId5"/>
+    <sheet name="สรุปรวมปี_2569" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="146">
   <si>
     <t>รายงานสรุปผลประกอบการ ร้านลูกชิ้น (19 วันแรก กันยายน 2569)</t>
   </si>
@@ -371,6 +372,102 @@
   </si>
   <si>
     <t>ยอดขายและกำไรสุทธิอันดับ 1 ของทุกสาขา (กำไรสะสม +42,801 บ.)</t>
+  </si>
+  <si>
+    <t>สรุปภาพรวมผลประกอบการประจำปี 2569 (มกราคม - กันยายน 2569)</t>
+  </si>
+  <si>
+    <t>ข้อมูลสังเคราะห์ทั้ง 4 สาขา (ยอดขายรวมทะลุ 1,079,924 บาท • กำไรสุทธิรวมเป็นบวก)</t>
+  </si>
+  <si>
+    <t>1. ตารางสรุปเปรียบเทียบผลประกอบการ 4 สาขา ประจำปี 2569</t>
+  </si>
+  <si>
+    <t>ช่วงเวลาบันทึก</t>
+  </si>
+  <si>
+    <t>สัดส่วนรายรับ</t>
+  </si>
+  <si>
+    <t>สถานะ / บทบาทธุรกิจ</t>
+  </si>
+  <si>
+    <t>9 เดือน (ม.ค.-ก.ย.)</t>
+  </si>
+  <si>
+    <t>Cash Cow อันดับ 1 (กำไรสูงสุด +42,801 บ. ยอดขายสูงสุด)</t>
+  </si>
+  <si>
+    <t>ก.ย. (19 วันแรก)</t>
+  </si>
+  <si>
+    <t>บันทึก 19 วันแรก ก.ย. (ค่าเช่ารอบ 3 ด. เฉลี่ย 3,333 บ./ด.)</t>
+  </si>
+  <si>
+    <t>ยอดขายสม่ำเสมออันดับ 2 ทะลุเป้า 40k ติดกัน 4 เดือนซ้อน</t>
+  </si>
+  <si>
+    <t>7 เดือน (มี.ค.-ก.ย.)</t>
+  </si>
+  <si>
+    <t>เติบโตเร็วที่สุด (+72% MoM) ค่าเช่ารอบ 3 เดือน</t>
+  </si>
+  <si>
+    <t>รวมทั้งกิจการ</t>
+  </si>
+  <si>
+    <t>ม.ค. - ก.ย. 2569</t>
+  </si>
+  <si>
+    <t>ยอดขายทะลุ 1.07 ล้านบาท พลิกกลับมามีกำไรสุทธิรวมทั้งกิจการ</t>
+  </si>
+  <si>
+    <t>2. ตารางสรุปผลประกอบการรายเดือนทั้งกิจการ (มกราคม - กันยายน 2569)</t>
+  </si>
+  <si>
+    <t>สาขา 1 (บาท)</t>
+  </si>
+  <si>
+    <t>สาขา 2 (บาท)</t>
+  </si>
+  <si>
+    <t>สาขา 3 (บาท)</t>
+  </si>
+  <si>
+    <t>สาขา 4 (บาท)</t>
+  </si>
+  <si>
+    <t>รายรับรวม (บาท)</t>
+  </si>
+  <si>
+    <t>เปิดปีใหม่ ยอดขายทะลุ 1.2 แสน สาขา 3 ทำ All-Time High 7.7 หมื่น</t>
+  </si>
+  <si>
+    <t>เดือนสั้น 28 วัน ยอดชะลอตัว</t>
+  </si>
+  <si>
+    <t>สาขา 4 เปิดขายเดือนแรก ยอดรวมแตะ 1.09 แสนบาท</t>
+  </si>
+  <si>
+    <t>All-Time High! เทศกาลสงกรานต์ ยอดพุ่งทะลุ 2 แสน กำไรสุทธิ +4.4 หมื่น</t>
+  </si>
+  <si>
+    <t>สาขา 4 ทะลุเป้า 30k ยอดรวมเกิน 1.08 แสน กำไรสุทธิเป็นบวก</t>
+  </si>
+  <si>
+    <t>ต้นฤดูฝน มีรอบจ่ายค่าเช่าและสต็อกของหลายสาขา</t>
+  </si>
+  <si>
+    <t>ยอดขายฟื้นตัวแข็งแกร่ง ทุกสาขาเติบโตแตะ 1.4 แสนบาท</t>
+  </si>
+  <si>
+    <t>สาขา 4 ทำ ATH พลิกกลับมามีกำไรสุทธิรวม +4,681 บ.</t>
+  </si>
+  <si>
+    <t>ข้อมูล 19 วันแรก รวม 4 สาขา คาดสิ้นเดือนทะลุ 1.4 แสนบาท</t>
+  </si>
+  <si>
+    <t>ยอดขายรวมทั้งปี 1,079,924 บ. กำไรสุทธิรวมเป็นบวก</t>
   </si>
 </sst>
 </file>
@@ -380,7 +477,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -450,8 +547,47 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF475569"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF312E81"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -506,6 +642,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0E7FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC7D2FE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -530,7 +690,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -567,9 +727,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -593,6 +750,36 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="1" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -921,15 +1108,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1983,17 +2170,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -2709,49 +2896,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="29" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2775,11 +2962,11 @@
         <v>5639</v>
       </c>
       <c r="G4" s="4">
-        <f>D4-E4</f>
+        <f t="shared" ref="G4:G14" si="0">D4-E4</f>
         <v>13026</v>
       </c>
       <c r="H4" s="5">
-        <f>G4/D4</f>
+        <f t="shared" ref="H4:H14" si="1">G4/D4</f>
         <v>0.29112933866750107</v>
       </c>
       <c r="I4" s="17" t="s">
@@ -2806,11 +2993,11 @@
         <v>5000</v>
       </c>
       <c r="G5" s="4">
-        <f>D5-E5</f>
+        <f t="shared" si="0"/>
         <v>913</v>
       </c>
       <c r="H5" s="5">
-        <f>G5/D5</f>
+        <f t="shared" si="1"/>
         <v>2.8974928594097112E-2</v>
       </c>
       <c r="I5" s="17" t="s">
@@ -2837,11 +3024,11 @@
         <v>5000</v>
       </c>
       <c r="G6" s="4">
-        <f>D6-E6</f>
+        <f t="shared" si="0"/>
         <v>-2894</v>
       </c>
       <c r="H6" s="5">
-        <f>G6/D6</f>
+        <f t="shared" si="1"/>
         <v>-5.3224946204917883E-2</v>
       </c>
       <c r="I6" s="17" t="s">
@@ -2868,11 +3055,11 @@
         <v>5000</v>
       </c>
       <c r="G7" s="4">
-        <f>D7-E7</f>
+        <f t="shared" si="0"/>
         <v>45056</v>
       </c>
       <c r="H7" s="5">
-        <f>G7/D7</f>
+        <f t="shared" si="1"/>
         <v>0.31242242485178379</v>
       </c>
       <c r="I7" s="17" t="s">
@@ -2899,11 +3086,11 @@
         <v>5000</v>
       </c>
       <c r="G8" s="4">
-        <f>D8-E8</f>
+        <f t="shared" si="0"/>
         <v>-1756</v>
       </c>
       <c r="H8" s="5">
-        <f>G8/D8</f>
+        <f t="shared" si="1"/>
         <v>-3.8798055678303141E-2</v>
       </c>
       <c r="I8" s="17" t="s">
@@ -2930,11 +3117,11 @@
         <v>7554</v>
       </c>
       <c r="G9" s="4">
-        <f>D9-E9</f>
+        <f t="shared" si="0"/>
         <v>-13953</v>
       </c>
       <c r="H9" s="5">
-        <f>G9/D9</f>
+        <f t="shared" si="1"/>
         <v>-0.41944987223808811</v>
       </c>
       <c r="I9" s="17" t="s">
@@ -2961,11 +3148,11 @@
         <v>5000</v>
       </c>
       <c r="G10" s="4">
-        <f>D10-E10</f>
+        <f t="shared" si="0"/>
         <v>349</v>
       </c>
       <c r="H10" s="5">
-        <f>G10/D10</f>
+        <f t="shared" si="1"/>
         <v>6.1912364733014017E-3</v>
       </c>
       <c r="I10" s="17" t="s">
@@ -2992,11 +3179,11 @@
         <v>2150</v>
       </c>
       <c r="G11" s="4">
-        <f>D11-E11</f>
+        <f t="shared" si="0"/>
         <v>4333</v>
       </c>
       <c r="H11" s="5">
-        <f>G11/D11</f>
+        <f t="shared" si="1"/>
         <v>9.8466083399613685E-2</v>
       </c>
       <c r="I11" s="17" t="s">
@@ -3023,11 +3210,11 @@
         <v>5000</v>
       </c>
       <c r="G12" s="4">
-        <f>D12-E12</f>
+        <f t="shared" si="0"/>
         <v>-2273</v>
       </c>
       <c r="H12" s="5">
-        <f>G12/D12</f>
+        <f t="shared" si="1"/>
         <v>-0.11526369168356998</v>
       </c>
       <c r="I12" s="17" t="s">
@@ -3035,70 +3222,821 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="23">
         <f>SUM(D4:D12)</f>
         <v>473461</v>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="23">
         <f>SUM(E4:E12)</f>
         <v>430660</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="23">
         <f>SUM(F4:F12)</f>
         <v>45343</v>
       </c>
-      <c r="G13" s="24">
-        <f>D13-E13</f>
+      <c r="G13" s="23">
+        <f t="shared" si="0"/>
         <v>42801</v>
       </c>
-      <c r="H13" s="26">
-        <f>G13/D13</f>
+      <c r="H13" s="25">
+        <f t="shared" si="1"/>
         <v>9.0400265280561651E-2</v>
       </c>
-      <c r="I13" s="31" t="s">
+      <c r="I13" s="30" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="25">
+      <c r="D14" s="24">
         <f>AVERAGE(D4:D12)</f>
         <v>52606.777777777781</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="24">
         <f>AVERAGE(E4:E12)</f>
         <v>47851.111111111109</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="24">
         <f>AVERAGE(F4:F12)</f>
         <v>5038.1111111111113</v>
       </c>
-      <c r="G14" s="25">
-        <f>D14-E14</f>
+      <c r="G14" s="24">
+        <f t="shared" si="0"/>
         <v>4755.6666666666715</v>
       </c>
-      <c r="H14" s="27">
-        <f>G14/D14</f>
+      <c r="H14" s="26">
+        <f t="shared" si="1"/>
         <v>9.0400265280561734E-2</v>
       </c>
-      <c r="I14" s="32" t="s">
+      <c r="I14" s="31" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDF6D89C-DDE2-4B0B-8F3D-FCE090BADFF6}">
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="89.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="61.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
+      <c r="A1" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="34" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="35" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="K5" s="36" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" s="4">
+        <v>370000</v>
+      </c>
+      <c r="D6" s="4">
+        <v>473461</v>
+      </c>
+      <c r="E6" s="5">
+        <f>D6/$D$10</f>
+        <v>0.43842066663950424</v>
+      </c>
+      <c r="F6" s="4">
+        <v>385317</v>
+      </c>
+      <c r="G6" s="4">
+        <v>45343</v>
+      </c>
+      <c r="H6" s="4">
+        <f>F6+G6</f>
+        <v>430660</v>
+      </c>
+      <c r="I6" s="4">
+        <f>D6-H6</f>
+        <v>42801</v>
+      </c>
+      <c r="J6" s="5">
+        <f>I6/D6</f>
+        <v>9.0400265280561651E-2</v>
+      </c>
+      <c r="K6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="4">
+        <v>40000</v>
+      </c>
+      <c r="D7" s="4">
+        <v>19890</v>
+      </c>
+      <c r="E7" s="5">
+        <f>D7/$D$10</f>
+        <v>1.8417962745526536E-2</v>
+      </c>
+      <c r="F7" s="4">
+        <v>25260</v>
+      </c>
+      <c r="G7" s="4">
+        <v>3333.33</v>
+      </c>
+      <c r="H7" s="4">
+        <f>F7+G7</f>
+        <v>28593.33</v>
+      </c>
+      <c r="I7" s="4">
+        <f>D7-H7</f>
+        <v>-8703.3300000000017</v>
+      </c>
+      <c r="J7" s="5">
+        <f>I7/D7</f>
+        <v>-0.43757315233785832</v>
+      </c>
+      <c r="K7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="4">
+        <v>400000</v>
+      </c>
+      <c r="D8" s="4">
+        <v>387155</v>
+      </c>
+      <c r="E8" s="5">
+        <f>D8/$D$10</f>
+        <v>0.35850207977598425</v>
+      </c>
+      <c r="F8" s="4">
+        <v>387569</v>
+      </c>
+      <c r="G8" s="4">
+        <v>24000</v>
+      </c>
+      <c r="H8" s="4">
+        <f>F8+G8</f>
+        <v>411569</v>
+      </c>
+      <c r="I8" s="4">
+        <f>D8-H8</f>
+        <v>-24414</v>
+      </c>
+      <c r="J8" s="5">
+        <f>I8/D8</f>
+        <v>-6.3060014722785454E-2</v>
+      </c>
+      <c r="K8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="4">
+        <v>230000</v>
+      </c>
+      <c r="D9" s="4">
+        <v>199418</v>
+      </c>
+      <c r="E9" s="5">
+        <f>D9/$D$10</f>
+        <v>0.18465929083898497</v>
+      </c>
+      <c r="F9" s="4">
+        <v>194817</v>
+      </c>
+      <c r="G9" s="4">
+        <v>13335.99</v>
+      </c>
+      <c r="H9" s="4">
+        <f>F9+G9</f>
+        <v>208152.99</v>
+      </c>
+      <c r="I9" s="4">
+        <f>D9-H9</f>
+        <v>-8734.9899999999907</v>
+      </c>
+      <c r="J9" s="5">
+        <f>I9/D9</f>
+        <v>-4.3802415027730648E-2</v>
+      </c>
+      <c r="K9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="38">
+        <f>SUM(C6:C9)</f>
+        <v>1040000</v>
+      </c>
+      <c r="D10" s="38">
+        <f>SUM(D6:D9)</f>
+        <v>1079924</v>
+      </c>
+      <c r="E10" s="39">
+        <f>SUM(E6:E9)</f>
+        <v>1</v>
+      </c>
+      <c r="F10" s="38">
+        <f>SUM(F6:F9)</f>
+        <v>992963</v>
+      </c>
+      <c r="G10" s="38">
+        <f>SUM(G6:G9)</f>
+        <v>86012.32</v>
+      </c>
+      <c r="H10" s="38">
+        <f>SUM(H6:H9)</f>
+        <v>1078975.32</v>
+      </c>
+      <c r="I10" s="38">
+        <f>SUM(I6:I9)</f>
+        <v>948.68000000000757</v>
+      </c>
+      <c r="J10" s="39">
+        <f>I10/D10</f>
+        <v>8.7846922561217976E-4</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="35" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="41" t="s">
+        <v>131</v>
+      </c>
+      <c r="D13" s="41" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" s="41" t="s">
+        <v>133</v>
+      </c>
+      <c r="F13" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="G13" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="H13" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="J13" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="K13" s="41" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C14" s="4">
+        <v>44743</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>77494</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <f>SUM(C14)</f>
+        <v>44743</v>
+      </c>
+      <c r="H14" s="4">
+        <v>97468</v>
+      </c>
+      <c r="I14" s="4">
+        <f>G14-H14</f>
+        <v>-52725</v>
+      </c>
+      <c r="J14" s="5">
+        <f>I14/G14</f>
+        <v>-1.1783966207004448</v>
+      </c>
+      <c r="K14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C15" s="4">
+        <v>31510</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>44473</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
+        <f>SUM(C15)</f>
+        <v>31510</v>
+      </c>
+      <c r="H15" s="4">
+        <v>89714</v>
+      </c>
+      <c r="I15" s="4">
+        <f>G15-H15</f>
+        <v>-58204</v>
+      </c>
+      <c r="J15" s="5">
+        <f>I15/G15</f>
+        <v>-1.8471596318629007</v>
+      </c>
+      <c r="K15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C16" s="4">
+        <v>54373</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4">
+        <v>32186</v>
+      </c>
+      <c r="F16" s="4">
+        <v>22454</v>
+      </c>
+      <c r="G16" s="4">
+        <f>SUM(C16)</f>
+        <v>54373</v>
+      </c>
+      <c r="H16" s="4">
+        <v>121197</v>
+      </c>
+      <c r="I16" s="4">
+        <f>G16-H16</f>
+        <v>-66824</v>
+      </c>
+      <c r="J16" s="5">
+        <f>I16/G16</f>
+        <v>-1.2289923307523956</v>
+      </c>
+      <c r="K16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C17" s="4">
+        <v>144215</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4">
+        <v>37470</v>
+      </c>
+      <c r="F17" s="4">
+        <v>24236</v>
+      </c>
+      <c r="G17" s="4">
+        <f>SUM(C17)</f>
+        <v>144215</v>
+      </c>
+      <c r="H17" s="4">
+        <v>161200</v>
+      </c>
+      <c r="I17" s="4">
+        <f>G17-H17</f>
+        <v>-16985</v>
+      </c>
+      <c r="J17" s="5">
+        <f>I17/G17</f>
+        <v>-0.11777554345941824</v>
+      </c>
+      <c r="K17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C18" s="4">
+        <v>45260</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4">
+        <v>32214</v>
+      </c>
+      <c r="F18" s="4">
+        <v>31466</v>
+      </c>
+      <c r="G18" s="4">
+        <f>SUM(C18)</f>
+        <v>45260</v>
+      </c>
+      <c r="H18" s="4">
+        <v>108101</v>
+      </c>
+      <c r="I18" s="4">
+        <f>G18-H18</f>
+        <v>-62841</v>
+      </c>
+      <c r="J18" s="5">
+        <f>I18/G18</f>
+        <v>-1.38844454264251</v>
+      </c>
+      <c r="K18" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C19" s="4">
+        <v>33265</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4">
+        <v>41143</v>
+      </c>
+      <c r="F19" s="4">
+        <v>28368</v>
+      </c>
+      <c r="G19" s="4">
+        <f>SUM(C19)</f>
+        <v>33265</v>
+      </c>
+      <c r="H19" s="4">
+        <v>127963</v>
+      </c>
+      <c r="I19" s="4">
+        <f>G19-H19</f>
+        <v>-94698</v>
+      </c>
+      <c r="J19" s="5">
+        <f>I19/G19</f>
+        <v>-2.8467758905756799</v>
+      </c>
+      <c r="K19" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C20" s="4">
+        <v>56370</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="4">
+        <v>49295</v>
+      </c>
+      <c r="F20" s="4">
+        <v>34810</v>
+      </c>
+      <c r="G20" s="4">
+        <f>SUM(C20)</f>
+        <v>56370</v>
+      </c>
+      <c r="H20" s="4">
+        <v>142490</v>
+      </c>
+      <c r="I20" s="4">
+        <f>G20-H20</f>
+        <v>-86120</v>
+      </c>
+      <c r="J20" s="5">
+        <f>I20/G20</f>
+        <v>-1.5277629945006208</v>
+      </c>
+      <c r="K20" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C21" s="4">
+        <v>44005</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4">
+        <v>45812</v>
+      </c>
+      <c r="F21" s="4">
+        <v>38655</v>
+      </c>
+      <c r="G21" s="4">
+        <f>SUM(C21)</f>
+        <v>44005</v>
+      </c>
+      <c r="H21" s="4">
+        <v>123791</v>
+      </c>
+      <c r="I21" s="4">
+        <f>G21-H21</f>
+        <v>-79786</v>
+      </c>
+      <c r="J21" s="5">
+        <f>I21/G21</f>
+        <v>-1.8131121463470061</v>
+      </c>
+      <c r="K21" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" s="13">
+        <v>2569</v>
+      </c>
+      <c r="C22" s="4">
+        <v>19720</v>
+      </c>
+      <c r="D22" s="4">
+        <v>19890</v>
+      </c>
+      <c r="E22" s="4">
+        <v>27068</v>
+      </c>
+      <c r="F22" s="4">
+        <v>23885</v>
+      </c>
+      <c r="G22" s="4">
+        <f>SUM(C22)</f>
+        <v>19720</v>
+      </c>
+      <c r="H22" s="4">
+        <v>107051</v>
+      </c>
+      <c r="I22" s="4">
+        <f>G22-H22</f>
+        <v>-87331</v>
+      </c>
+      <c r="J22" s="5">
+        <f>I22/G22</f>
+        <v>-4.4285496957403652</v>
+      </c>
+      <c r="K22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="48" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="48" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="44">
+        <f>SUM(C14:C22)</f>
+        <v>473461</v>
+      </c>
+      <c r="D23" s="44">
+        <f>SUM(D14:D22)</f>
+        <v>19890</v>
+      </c>
+      <c r="E23" s="44">
+        <f>SUM(E14:E22)</f>
+        <v>387155</v>
+      </c>
+      <c r="F23" s="44">
+        <f>SUM(F14:F22)</f>
+        <v>203874</v>
+      </c>
+      <c r="G23" s="44">
+        <f>SUM(G14:G22)</f>
+        <v>473461</v>
+      </c>
+      <c r="H23" s="44">
+        <f>SUM(H14:H22)</f>
+        <v>1078975</v>
+      </c>
+      <c r="I23" s="44">
+        <f>G23-H23</f>
+        <v>-605514</v>
+      </c>
+      <c r="J23" s="46">
+        <f>I23/G23</f>
+        <v>-1.2789099841380811</v>
+      </c>
+      <c r="K23" s="42" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="49" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" s="49" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="45">
+        <f>AVERAGE(C14:C22)</f>
+        <v>52606.777777777781</v>
+      </c>
+      <c r="D24" s="45">
+        <f>AVERAGE(D14:D22)</f>
+        <v>2210</v>
+      </c>
+      <c r="E24" s="45">
+        <f>AVERAGE(E14:E22)</f>
+        <v>43017.222222222219</v>
+      </c>
+      <c r="F24" s="45">
+        <f>AVERAGE(F14:F22)</f>
+        <v>22652.666666666668</v>
+      </c>
+      <c r="G24" s="45">
+        <f>AVERAGE(G14:G22)</f>
+        <v>52606.777777777781</v>
+      </c>
+      <c r="H24" s="45">
+        <f>AVERAGE(H14:H22)</f>
+        <v>119886.11111111111</v>
+      </c>
+      <c r="I24" s="45">
+        <f>G24-H24</f>
+        <v>-67279.333333333328</v>
+      </c>
+      <c r="J24" s="47">
+        <f>I24/G24</f>
+        <v>-1.2789099841380809</v>
+      </c>
+      <c r="K24" s="43" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>